<commit_message>
Rename project label text
Co-authored-by: Davevw <157815766+Davevw@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/public/assets/HoustonITP_CapitalModel_v1.xlsx
+++ b/public/assets/HoustonITP_CapitalModel_v1.xlsx
@@ -521,7 +521,7 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>International Freight Park Houston (ITPH)</t>
+          <t>International Trade Park Houston (ITPH)</t>
         </is>
       </c>
     </row>
@@ -1152,7 +1152,7 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>This is the Houston ITP Capital Model — International Freight Park Houston</t>
+          <t>This is the Houston ITP Capital Model — International Trade Park Houston</t>
         </is>
       </c>
     </row>

</xml_diff>